<commit_message>
-Updated GERMANY_ECONOMIC_IMPORTANCE_SECTORS sector shares to match each year's data per BGR Rohstoffsituationbericht (used USGS MCS if BGR data was N/A). -Corrected Comtrade csv files to fix country spelling errors. -Corrected Reserves.xlsx files for materials with missing world totals. -Re-ran refined model for 2017, 2020-2024; saved all refined results (replaced older results).
</commit_message>
<xml_diff>
--- a/Data point Supporting files/Germany 2017 (new)/Reserves.xlsx
+++ b/Data point Supporting files/Germany 2017 (new)/Reserves.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="31"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="27"/>
   </bookViews>
   <sheets>
     <sheet name="Aluminium" sheetId="1" state="visible" r:id="rId2"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="171">
   <si>
     <t xml:space="preserve">Country</t>
   </si>
@@ -648,7 +648,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -658,14 +658,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1112,7 +1104,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -1450,7 +1442,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B44"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
@@ -2424,7 +2416,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B101"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
@@ -2575,18 +2567,18 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="0" t="n">
         <v>108000000000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="1" t="n">
         <v>4000000000</v>
       </c>
     </row>
@@ -3087,106 +3079,106 @@
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="3" t="s">
+      <c r="A83" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B83" s="3" t="n">
+      <c r="B83" s="1" t="n">
         <v>215200000000</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="4" t="s">
+      <c r="A84" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="B84" s="4" t="n">
+      <c r="B84" s="0" t="n">
         <v>4800000000</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="4" t="s">
+      <c r="A85" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="B85" s="4" t="n">
+      <c r="B85" s="0" t="n">
         <v>4800000000</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="4" t="s">
+      <c r="A86" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="B86" s="4" t="n">
+      <c r="B86" s="0" t="n">
         <v>29600000000</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="4" t="s">
+      <c r="A87" s="0" t="s">
         <v>125</v>
       </c>
-      <c r="B87" s="4" t="n">
+      <c r="B87" s="0" t="n">
         <v>160000000000</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="4" t="s">
+      <c r="A88" s="0" t="s">
         <v>127</v>
       </c>
-      <c r="B88" s="4" t="n">
+      <c r="B88" s="0" t="n">
         <v>208000000000</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="4" t="s">
+      <c r="A89" s="0" t="s">
         <v>128</v>
       </c>
-      <c r="B89" s="4" t="n">
+      <c r="B89" s="0" t="n">
         <v>52000000000</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="4" t="s">
+      <c r="A90" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="B90" s="4" t="n">
+      <c r="B90" s="0" t="n">
         <v>4000000000</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="4" t="s">
+      <c r="A91" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="B91" s="4" t="n">
+      <c r="B91" s="0" t="n">
         <v>7870400000000</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="4" t="s">
+      <c r="A92" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="B92" s="4" t="n">
+      <c r="B92" s="0" t="n">
         <v>7253600000000</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="4" t="s">
+      <c r="A93" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="B93" s="4" t="n">
+      <c r="B93" s="0" t="n">
         <v>11200000000</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="4" t="s">
+      <c r="A94" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="B94" s="4" t="n">
+      <c r="B94" s="0" t="n">
         <v>760000000000</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="3" t="s">
+      <c r="A95" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B95" s="3" t="n">
+      <c r="B95" s="1" t="n">
         <v>4751200000000</v>
       </c>
     </row>
@@ -4091,7 +4083,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4102,11 +4094,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>6800000</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B3" s="1" t="n">
         <v>6800000</v>
       </c>
     </row>
@@ -4595,7 +4595,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
@@ -4666,34 +4666,34 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="1" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="0" t="n">
         <v>108000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="1" t="n">
         <v>18000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="0" t="n">
         <v>14000</v>
       </c>
     </row>
@@ -5281,7 +5281,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B70"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
@@ -5447,11 +5447,11 @@
         <v>201000000</v>
       </c>
     </row>
-    <row r="21" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="1" t="n">
         <v>3000000</v>
       </c>
     </row>
@@ -6126,7 +6126,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B107"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>

</xml_diff>